<commit_message>
F-52: typo-tolerant client names
</commit_message>
<xml_diff>
--- a/Agent_Fix_Tracker.xlsx
+++ b/Agent_Fix_Tracker.xlsx
@@ -15,8 +15,8 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Decide &amp; Next'!$A$1:$J$18</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Fixes!$A$1:$N$52</definedName>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Tests!$A$1:$M$97</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Fixes!$A$1:$N$53</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Tests!$A$1:$M$102</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1626" uniqueCount="865">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1679" uniqueCount="891">
   <si>
     <t xml:space="preserve">Debit Card Agent — Fix Tracker</t>
   </si>
@@ -96,7 +96,7 @@
     <t xml:space="preserve">Pass</t>
   </si>
   <si>
-    <t xml:space="preserve">Round 3 (Oct 24): F-47 to F-51 come from pending_fixes_2 P2-01 to P2-05.</t>
+    <t xml:space="preserve">Round 3 (Oct 24-25): F-47 to F-52 come from pending_fixes_2 P2-01 to P2-06.</t>
   </si>
   <si>
     <t xml:space="preserve">Fail</t>
@@ -1215,6 +1215,24 @@
     <t xml:space="preserve">Code reads an address typed in the message: outside the US -&gt; said above the field; US -&gt; put in the field so the suggestions show at once.</t>
   </si>
   <si>
+    <t xml:space="preserve">F-52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capitals and small typos in the client's name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Names with typos or swapped letters were not recognised (P2-06)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guy, Oct 25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-52a, T-52b, T-52c, T-52d, T-52e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Names are matched without regard to capitals; small typos and swapped letters (1 letter off in short names, 2 in longer ones) get 'Did you mean ...?' Yes / Another client / Cancel. Only this advisor's clients are considered.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Type</t>
   </si>
   <si>
@@ -1404,7 +1422,7 @@
     <t xml:space="preserve">R-06</t>
   </si>
   <si>
-    <t xml:space="preserve">Run the round 3 tests (T-47a to T-51b) and T-10a, T-28a, T-28f again</t>
+    <t xml:space="preserve">Run the round 3 tests (T-47a to T-52e) and T-10a, T-28a, T-28f again</t>
   </si>
   <si>
     <t xml:space="preserve">Fixed in round 3 (F-47 to F-51)</t>
@@ -2590,6 +2608,66 @@
   </si>
   <si>
     <t xml:space="preserve">The field already holds '1100 Congress Ave, Austin' with suggestions showing; pick, Use this address, then the red card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-52a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any capitalisation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOCK JANE MILLER'S CARD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jane Miller found; lock card shown, no extra question.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-52b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typo in the name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lock Jnae Millre's card → Yes, Jane Miller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Did you mean Jane Miller (New York, born 1979)?' Yes / Another client / Cancel. Yes: the lock card.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-52c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typo, lower case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lock robert castelano card</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Did you mean Robert Castellano (Greenwich, born 1961)?'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-52d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typo matching several clients</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lock sara chen card</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Did you mean one of these?' with both Sarah Chens as buttons.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-52e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typo never reveals other advisors' clients</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lock Jnae Millre's card</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'No client named Jnae Millre was found.' Jane Miller is never suggested.</t>
   </si>
   <si>
     <t xml:space="preserve">T-R01</t>
@@ -3406,7 +3484,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">COUNTIF(Fixes!J2:J300,"Fixed")</f>
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>9</v>
@@ -3442,7 +3520,7 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">SUM(B5:B9)</f>
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>15</v>
@@ -3467,7 +3545,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">COUNTIF(Tests!I2:I300,"Not run")</f>
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>20</v>
@@ -3509,7 +3587,7 @@
       </c>
       <c r="B17" s="6" t="n">
         <f aca="false">SUM(B13:B16)</f>
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3523,7 +3601,7 @@
       </c>
       <c r="B20" s="6" t="n">
         <f aca="false">COUNTIF(Tests!H2:H300,"Pass")</f>
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3550,7 +3628,7 @@
       </c>
       <c r="B23" s="6" t="n">
         <f aca="false">SUM(B20:B22)</f>
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3619,7 +3697,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -5867,9 +5945,53 @@
         <v>394</v>
       </c>
     </row>
+    <row r="53" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="B53" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>396</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>397</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="F53" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="G53" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="H53" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="I53" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="J53" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="K53" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L53" s="12" t="n">
+        <v>46319</v>
+      </c>
+      <c r="M53" s="10" t="s">
+        <v>399</v>
+      </c>
+      <c r="N53" s="11" t="s">
+        <v>400</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N52"/>
-  <conditionalFormatting sqref="J2:J252">
+  <autoFilter ref="A1:N53"/>
+  <conditionalFormatting sqref="J2:J253">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$J2="Verified"</formula>
     </cfRule>
@@ -5886,7 +6008,7 @@
       <formula>$J2="Not started"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F252">
+  <conditionalFormatting sqref="F2:F253">
     <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$F2="High"</formula>
     </cfRule>
@@ -5898,19 +6020,19 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J2:J252" type="list">
+    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J2:J253" type="list">
       <formula1>"Not started,In progress,Fixed,Verified,Blocked"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F252" type="list">
+    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F253" type="list">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G2:G252" type="list">
+    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G2:G253" type="list">
       <formula1>"Easy,Medium,Hard"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B2:B252" type="list">
+    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B2:B253" type="list">
       <formula1>"Rule in code,Prompt,Message,UX,Feature"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5951,31 +6073,31 @@
         <v>33</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>42</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5983,25 +6105,25 @@
         <v>54</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="G2" s="11" t="s">
         <v>29</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="I2" s="12"/>
       <c r="J2" s="11"/>
@@ -6011,25 +6133,25 @@
         <v>70</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="G3" s="11" t="s">
         <v>32</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
       <c r="I3" s="12" t="n">
         <v>46319</v>
@@ -6041,16 +6163,16 @@
         <v>93</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>88</v>
@@ -6059,29 +6181,29 @@
         <v>29</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="I4" s="12"/>
       <c r="J4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>29</v>
@@ -6095,16 +6217,16 @@
         <v>162</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="F6" s="10" t="s">
         <v>159</v>
@@ -6113,7 +6235,7 @@
         <v>32</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="I6" s="12" t="n">
         <v>46319</v>
@@ -6125,16 +6247,16 @@
         <v>107</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="F7" s="10" t="s">
         <v>103</v>
@@ -6143,35 +6265,35 @@
         <v>29</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>32</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="I8" s="12" t="n">
         <v>46319</v>
@@ -6180,28 +6302,28 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>439</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>433</v>
-      </c>
       <c r="C9" s="10" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>32</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
       <c r="I9" s="12" t="n">
         <v>46319</v>
@@ -6210,28 +6332,28 @@
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
+        <v>449</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>439</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>451</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>452</v>
+      </c>
+      <c r="F10" s="10" t="s">
         <v>443</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>433</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>445</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>446</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>437</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>32</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="I10" s="12" t="n">
         <v>46319</v>
@@ -6240,50 +6362,50 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>29</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="I11" s="12"/>
       <c r="J11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="G12" s="11" t="s">
         <v>29</v>
@@ -6294,22 +6416,22 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="G13" s="11" t="s">
         <v>29</v>
@@ -6320,22 +6442,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="G14" s="11" t="s">
         <v>29</v>
@@ -6346,22 +6468,22 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="G15" s="11" t="s">
         <v>29</v>
@@ -6372,22 +6494,22 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="G16" s="11" t="s">
         <v>29</v>
@@ -6398,22 +6520,22 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="G17" s="11" t="s">
         <v>29</v>
@@ -6424,22 +6546,22 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="G18" s="11" t="s">
         <v>29</v>
@@ -6504,7 +6626,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M97"/>
+  <dimension ref="A1:M102"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -6523,63 +6645,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="I1" s="14" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="J1" s="14" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="K1" s="14" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
       <c r="L1" s="14" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="M1" s="14" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>47</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="G2" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B2,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B2,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -6598,22 +6720,22 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>47</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="G3" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B3,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B3,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -6632,22 +6754,22 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>47</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="G4" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B4,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B4,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -6666,22 +6788,22 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>47</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="G5" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B5,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B5,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -6706,16 +6828,16 @@
         <v>59</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="G6" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B6,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B6,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -6734,22 +6856,22 @@
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="G7" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B7,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B7,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -6768,22 +6890,22 @@
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="G8" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B8,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B8,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -6799,27 +6921,27 @@
       <c r="K8" s="11"/>
       <c r="L8" s="12"/>
       <c r="M8" s="11" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="G9" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B9,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B9,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -6838,22 +6960,22 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="G10" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B10,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B10,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -6872,22 +6994,22 @@
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="G11" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B11,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B11,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -6906,22 +7028,22 @@
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>74</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="G12" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B12,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B12,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -6937,27 +7059,27 @@
       <c r="K12" s="11"/>
       <c r="L12" s="12"/>
       <c r="M12" s="11" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>74</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="G13" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B13,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B13,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -6976,22 +7098,22 @@
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>74</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="G14" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B14,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B14,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7010,22 +7132,22 @@
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>81</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="G15" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B15,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B15,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7041,27 +7163,27 @@
       <c r="K15" s="11"/>
       <c r="L15" s="12"/>
       <c r="M15" s="11" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>81</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="G16" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B16,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B16,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7080,22 +7202,22 @@
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>88</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="G17" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B17,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B17,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7111,27 +7233,27 @@
       <c r="K17" s="11"/>
       <c r="L17" s="12"/>
       <c r="M17" s="11" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>88</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="G18" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B18,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B18,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7147,7 +7269,7 @@
       <c r="K18" s="11"/>
       <c r="L18" s="12"/>
       <c r="M18" s="11" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7158,16 +7280,16 @@
         <v>96</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="G19" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B19,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B19,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7192,16 +7314,16 @@
         <v>103</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="G20" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B20,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B20,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7217,7 +7339,7 @@
       <c r="K20" s="11"/>
       <c r="L20" s="12"/>
       <c r="M20" s="11" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7228,16 +7350,16 @@
         <v>110</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="G21" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B21,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B21,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7262,16 +7384,16 @@
         <v>118</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="G22" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B22,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B22,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7287,27 +7409,27 @@
       <c r="K22" s="11"/>
       <c r="L22" s="12"/>
       <c r="M22" s="11" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>126</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="G23" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B23,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B23,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7326,22 +7448,22 @@
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>126</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="G24" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B24,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B24,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7360,22 +7482,22 @@
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>133</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="G25" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B25,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B25,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7394,22 +7516,22 @@
     </row>
     <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>133</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="G26" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B26,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B26,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7425,27 +7547,27 @@
       <c r="K26" s="11"/>
       <c r="L26" s="12"/>
       <c r="M26" s="11" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>139</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="G27" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B27,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B27,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7464,22 +7586,22 @@
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>139</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
       <c r="G28" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B28,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B28,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7504,16 +7626,16 @@
         <v>145</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="G29" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B29,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B29,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7529,7 +7651,7 @@
       <c r="K29" s="11"/>
       <c r="L29" s="12"/>
       <c r="M29" s="11" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7540,16 +7662,16 @@
         <v>152</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="G30" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B30,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B30,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7565,7 +7687,7 @@
       <c r="K30" s="11"/>
       <c r="L30" s="12"/>
       <c r="M30" s="11" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7576,16 +7698,16 @@
         <v>159</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="F31" s="10" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="G31" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B31,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B31,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7601,27 +7723,27 @@
       <c r="K31" s="11"/>
       <c r="L31" s="12"/>
       <c r="M31" s="11" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
       <c r="B32" s="10" t="s">
         <v>166</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="F32" s="10" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
       <c r="G32" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B32,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B32,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7640,22 +7762,22 @@
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>166</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
       <c r="F33" s="10" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="G33" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B33,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B33,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7680,16 +7802,16 @@
         <v>174</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
       <c r="F34" s="10" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="G34" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B34,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B34,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7714,16 +7836,16 @@
         <v>180</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
       <c r="G35" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B35,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B35,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7742,22 +7864,22 @@
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
       <c r="B36" s="10" t="s">
         <v>186</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
       <c r="F36" s="10" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
       <c r="G36" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B36,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B36,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7773,27 +7895,27 @@
       <c r="K36" s="11"/>
       <c r="L36" s="12"/>
       <c r="M36" s="11" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
       <c r="B37" s="10" t="s">
         <v>186</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="F37" s="10" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
       <c r="G37" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B37,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B37,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7809,27 +7931,27 @@
       <c r="K37" s="11"/>
       <c r="L37" s="12"/>
       <c r="M37" s="11" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>186</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="F38" s="10" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
       <c r="G38" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B38,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B38,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7845,27 +7967,27 @@
       <c r="K38" s="11"/>
       <c r="L38" s="12"/>
       <c r="M38" s="11" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
       <c r="B39" s="10" t="s">
         <v>186</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="G39" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B39,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B39,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7890,16 +8012,16 @@
         <v>193</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
       <c r="F40" s="10" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
       <c r="G40" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B40,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B40,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7915,7 +8037,7 @@
       <c r="K40" s="11"/>
       <c r="L40" s="12"/>
       <c r="M40" s="11" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7926,16 +8048,16 @@
         <v>199</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="F41" s="10" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="G41" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B41,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B41,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7951,7 +8073,7 @@
       <c r="K41" s="11"/>
       <c r="L41" s="12"/>
       <c r="M41" s="11" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7962,16 +8084,16 @@
         <v>205</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="F42" s="10" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="G42" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B42,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B42,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -7990,22 +8112,22 @@
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="B43" s="10" t="s">
         <v>212</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
       <c r="F43" s="10" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="G43" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B43,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B43,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8024,22 +8146,22 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
       <c r="B44" s="10" t="s">
         <v>212</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
       <c r="F44" s="10" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="G44" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B44,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B44,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8064,16 +8186,16 @@
         <v>219</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="G45" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B45,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B45,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8098,16 +8220,16 @@
         <v>224</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="F46" s="10" t="s">
-        <v>672</v>
+        <v>678</v>
       </c>
       <c r="G46" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B46,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B46,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8123,27 +8245,27 @@
       <c r="K46" s="11"/>
       <c r="L46" s="12"/>
       <c r="M46" s="11" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="9" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>230</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
       <c r="F47" s="10" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="G47" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B47,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B47,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8159,27 +8281,27 @@
       <c r="K47" s="11"/>
       <c r="L47" s="12"/>
       <c r="M47" s="11" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="9" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="B48" s="10" t="s">
         <v>230</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
       <c r="F48" s="10" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="G48" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B48,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B48,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8195,27 +8317,27 @@
       <c r="K48" s="11"/>
       <c r="L48" s="12"/>
       <c r="M48" s="11" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="9" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="B49" s="10" t="s">
         <v>230</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="F49" s="10" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
       <c r="G49" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B49,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B49,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8234,22 +8356,22 @@
     </row>
     <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="9" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="B50" s="10" t="s">
         <v>235</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="F50" s="10" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="G50" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B50,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B50,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8265,27 +8387,27 @@
       <c r="K50" s="11"/>
       <c r="L50" s="12"/>
       <c r="M50" s="11" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="9" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="B51" s="10" t="s">
         <v>235</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="F51" s="10" t="s">
-        <v>693</v>
+        <v>699</v>
       </c>
       <c r="G51" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B51,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B51,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8304,22 +8426,22 @@
     </row>
     <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="9" t="s">
-        <v>694</v>
+        <v>700</v>
       </c>
       <c r="B52" s="10" t="s">
         <v>235</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>696</v>
+        <v>702</v>
       </c>
       <c r="F52" s="10" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="G52" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B52,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B52,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8338,22 +8460,22 @@
     </row>
     <row r="53" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="9" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
       <c r="B53" s="10" t="s">
         <v>235</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>700</v>
+        <v>706</v>
       </c>
       <c r="F53" s="10" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
       <c r="G53" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B53,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B53,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8372,22 +8494,22 @@
     </row>
     <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
       <c r="B54" s="10" t="s">
         <v>235</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="D54" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>704</v>
+        <v>710</v>
       </c>
       <c r="F54" s="10" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="G54" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B54,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B54,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8406,22 +8528,22 @@
     </row>
     <row r="55" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="9" t="s">
-        <v>706</v>
+        <v>712</v>
       </c>
       <c r="B55" s="10" t="s">
         <v>235</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="F55" s="10" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="G55" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B55,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B55,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8437,27 +8559,27 @@
       <c r="K55" s="11"/>
       <c r="L55" s="12"/>
       <c r="M55" s="11" t="s">
-        <v>710</v>
+        <v>716</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="9" t="s">
-        <v>711</v>
+        <v>717</v>
       </c>
       <c r="B56" s="10" t="s">
         <v>235</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>712</v>
+        <v>718</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="F56" s="10" t="s">
-        <v>714</v>
+        <v>720</v>
       </c>
       <c r="G56" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B56,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B56,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8476,22 +8598,22 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="9" t="s">
-        <v>715</v>
+        <v>721</v>
       </c>
       <c r="B57" s="10" t="s">
         <v>235</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>716</v>
+        <v>722</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>717</v>
+        <v>723</v>
       </c>
       <c r="F57" s="10" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
       <c r="G57" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B57,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B57,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8510,22 +8632,22 @@
     </row>
     <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="9" t="s">
-        <v>719</v>
+        <v>725</v>
       </c>
       <c r="B58" s="10" t="s">
         <v>243</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>720</v>
+        <v>726</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>721</v>
+        <v>727</v>
       </c>
       <c r="F58" s="10" t="s">
-        <v>722</v>
+        <v>728</v>
       </c>
       <c r="G58" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B58,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B58,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8544,22 +8666,22 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="9" t="s">
-        <v>723</v>
+        <v>729</v>
       </c>
       <c r="B59" s="10" t="s">
         <v>243</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>725</v>
+        <v>731</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>726</v>
+        <v>732</v>
       </c>
       <c r="F59" s="10" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="G59" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B59,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B59,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8578,22 +8700,22 @@
     </row>
     <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="9" t="s">
-        <v>728</v>
+        <v>734</v>
       </c>
       <c r="B60" s="10" t="s">
         <v>243</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>729</v>
+        <v>735</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="F60" s="10" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
       <c r="G60" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B60,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B60,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8612,22 +8734,22 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="9" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="B61" s="10" t="s">
         <v>243</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
       <c r="F61" s="10" t="s">
-        <v>735</v>
+        <v>741</v>
       </c>
       <c r="G61" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B61,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B61,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8652,16 +8774,16 @@
         <v>250</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
       <c r="D62" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>737</v>
+        <v>743</v>
       </c>
       <c r="F62" s="10" t="s">
-        <v>738</v>
+        <v>744</v>
       </c>
       <c r="G62" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B62,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B62,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8680,22 +8802,22 @@
     </row>
     <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="9" t="s">
-        <v>739</v>
+        <v>745</v>
       </c>
       <c r="B63" s="10" t="s">
         <v>257</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>740</v>
+        <v>746</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>741</v>
+        <v>747</v>
       </c>
       <c r="F63" s="10" t="s">
-        <v>742</v>
+        <v>748</v>
       </c>
       <c r="G63" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B63,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B63,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8714,22 +8836,22 @@
     </row>
     <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="9" t="s">
-        <v>743</v>
+        <v>749</v>
       </c>
       <c r="B64" s="10" t="s">
         <v>257</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>744</v>
+        <v>750</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>745</v>
+        <v>751</v>
       </c>
       <c r="F64" s="10" t="s">
-        <v>746</v>
+        <v>752</v>
       </c>
       <c r="G64" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B64,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B64,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8754,16 +8876,16 @@
         <v>264</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>747</v>
+        <v>753</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>748</v>
+        <v>754</v>
       </c>
       <c r="F65" s="10" t="s">
-        <v>749</v>
+        <v>755</v>
       </c>
       <c r="G65" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B65,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B65,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8788,16 +8910,16 @@
         <v>271</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>750</v>
+        <v>756</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="F66" s="10" t="s">
-        <v>751</v>
+        <v>757</v>
       </c>
       <c r="G66" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B66,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B66,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8813,27 +8935,27 @@
       <c r="K66" s="11"/>
       <c r="L66" s="12"/>
       <c r="M66" s="11" t="s">
-        <v>752</v>
+        <v>758</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="9" t="s">
-        <v>753</v>
+        <v>759</v>
       </c>
       <c r="B67" s="10" t="s">
         <v>278</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>754</v>
+        <v>760</v>
       </c>
       <c r="D67" s="10" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>755</v>
+        <v>761</v>
       </c>
       <c r="F67" s="10" t="s">
-        <v>756</v>
+        <v>762</v>
       </c>
       <c r="G67" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B67,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B67,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8852,22 +8974,22 @@
     </row>
     <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="9" t="s">
-        <v>757</v>
+        <v>763</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>278</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>758</v>
+        <v>764</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>759</v>
+        <v>765</v>
       </c>
       <c r="F68" s="10" t="s">
-        <v>760</v>
+        <v>766</v>
       </c>
       <c r="G68" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B68,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B68,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8886,22 +9008,22 @@
     </row>
     <row r="69" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="9" t="s">
-        <v>761</v>
+        <v>767</v>
       </c>
       <c r="B69" s="10" t="s">
         <v>284</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>762</v>
+        <v>768</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="F69" s="10" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="G69" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B69,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B69,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8920,22 +9042,22 @@
     </row>
     <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="9" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="B70" s="10" t="s">
         <v>284</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
       <c r="D70" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>767</v>
+        <v>773</v>
       </c>
       <c r="F70" s="10" t="s">
-        <v>768</v>
+        <v>774</v>
       </c>
       <c r="G70" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B70,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B70,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8954,22 +9076,22 @@
     </row>
     <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="9" t="s">
-        <v>769</v>
+        <v>775</v>
       </c>
       <c r="B71" s="10" t="s">
         <v>291</v>
       </c>
       <c r="C71" s="10" t="s">
-        <v>770</v>
+        <v>776</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="F71" s="10" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
       <c r="G71" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B71,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B71,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -8988,22 +9110,22 @@
     </row>
     <row r="72" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="9" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="B72" s="10" t="s">
         <v>291</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>774</v>
+        <v>780</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>775</v>
+        <v>781</v>
       </c>
       <c r="F72" s="10" t="s">
-        <v>776</v>
+        <v>782</v>
       </c>
       <c r="G72" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B72,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B72,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9028,16 +9150,16 @@
         <v>298</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>778</v>
+        <v>784</v>
       </c>
       <c r="F73" s="10" t="s">
-        <v>779</v>
+        <v>785</v>
       </c>
       <c r="G73" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B73,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B73,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9062,16 +9184,16 @@
         <v>304</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>780</v>
+        <v>786</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>781</v>
+        <v>787</v>
       </c>
       <c r="F74" s="10" t="s">
-        <v>782</v>
+        <v>788</v>
       </c>
       <c r="G74" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B74,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B74,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9096,16 +9218,16 @@
         <v>312</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>784</v>
+        <v>790</v>
       </c>
       <c r="F75" s="10" t="s">
-        <v>785</v>
+        <v>791</v>
       </c>
       <c r="G75" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B75,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B75,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9130,16 +9252,16 @@
         <v>318</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>786</v>
+        <v>792</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>787</v>
+        <v>793</v>
       </c>
       <c r="F76" s="10" t="s">
-        <v>788</v>
+        <v>794</v>
       </c>
       <c r="G76" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B76,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B76,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9164,16 +9286,16 @@
         <v>325</v>
       </c>
       <c r="C77" s="10" t="s">
-        <v>789</v>
+        <v>795</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>790</v>
+        <v>796</v>
       </c>
       <c r="F77" s="10" t="s">
-        <v>791</v>
+        <v>797</v>
       </c>
       <c r="G77" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B77,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B77,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9198,16 +9320,16 @@
         <v>332</v>
       </c>
       <c r="C78" s="10" t="s">
-        <v>792</v>
+        <v>798</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>793</v>
+        <v>799</v>
       </c>
       <c r="F78" s="10" t="s">
-        <v>794</v>
+        <v>800</v>
       </c>
       <c r="G78" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B78,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B78,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9232,16 +9354,16 @@
         <v>338</v>
       </c>
       <c r="C79" s="10" t="s">
-        <v>795</v>
+        <v>801</v>
       </c>
       <c r="D79" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>796</v>
+        <v>802</v>
       </c>
       <c r="F79" s="10" t="s">
-        <v>797</v>
+        <v>803</v>
       </c>
       <c r="G79" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B79,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B79,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9260,22 +9382,22 @@
     </row>
     <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="9" t="s">
-        <v>798</v>
+        <v>804</v>
       </c>
       <c r="B80" s="10" t="s">
         <v>345</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>799</v>
+        <v>805</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>800</v>
+        <v>806</v>
       </c>
       <c r="F80" s="10" t="s">
-        <v>801</v>
+        <v>807</v>
       </c>
       <c r="G80" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B80,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B80,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9294,22 +9416,22 @@
     </row>
     <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="9" t="s">
-        <v>802</v>
+        <v>808</v>
       </c>
       <c r="B81" s="10" t="s">
         <v>345</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>803</v>
+        <v>809</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>804</v>
+        <v>810</v>
       </c>
       <c r="F81" s="10" t="s">
-        <v>805</v>
+        <v>811</v>
       </c>
       <c r="G81" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B81,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B81,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9334,16 +9456,16 @@
         <v>352</v>
       </c>
       <c r="C82" s="10" t="s">
-        <v>806</v>
+        <v>812</v>
       </c>
       <c r="D82" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>807</v>
+        <v>813</v>
       </c>
       <c r="F82" s="10" t="s">
-        <v>808</v>
+        <v>814</v>
       </c>
       <c r="G82" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B82,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B82,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9362,22 +9484,22 @@
     </row>
     <row r="83" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="9" t="s">
-        <v>809</v>
+        <v>815</v>
       </c>
       <c r="B83" s="10" t="s">
         <v>359</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>810</v>
+        <v>816</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>811</v>
+        <v>817</v>
       </c>
       <c r="F83" s="10" t="s">
-        <v>812</v>
+        <v>818</v>
       </c>
       <c r="G83" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B83,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B83,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9396,22 +9518,22 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="9" t="s">
-        <v>813</v>
+        <v>819</v>
       </c>
       <c r="B84" s="10" t="s">
         <v>359</v>
       </c>
       <c r="C84" s="10" t="s">
-        <v>814</v>
+        <v>820</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>815</v>
+        <v>821</v>
       </c>
       <c r="F84" s="10" t="s">
-        <v>816</v>
+        <v>822</v>
       </c>
       <c r="G84" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B84,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B84,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9430,22 +9552,22 @@
     </row>
     <row r="85" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="9" t="s">
-        <v>817</v>
+        <v>823</v>
       </c>
       <c r="B85" s="10" t="s">
         <v>365</v>
       </c>
       <c r="C85" s="10" t="s">
-        <v>818</v>
+        <v>824</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="F85" s="10" t="s">
-        <v>819</v>
+        <v>825</v>
       </c>
       <c r="G85" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B85,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B85,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9464,22 +9586,22 @@
     </row>
     <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="9" t="s">
-        <v>820</v>
+        <v>826</v>
       </c>
       <c r="B86" s="10" t="s">
         <v>365</v>
       </c>
       <c r="C86" s="10" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="D86" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>822</v>
+        <v>828</v>
       </c>
       <c r="F86" s="10" t="s">
-        <v>823</v>
+        <v>829</v>
       </c>
       <c r="G86" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B86,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B86,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9498,22 +9620,22 @@
     </row>
     <row r="87" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="9" t="s">
-        <v>824</v>
+        <v>830</v>
       </c>
       <c r="B87" s="10" t="s">
         <v>371</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>825</v>
+        <v>831</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
       <c r="F87" s="10" t="s">
-        <v>827</v>
+        <v>833</v>
       </c>
       <c r="G87" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B87,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B87,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9532,22 +9654,22 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="9" t="s">
-        <v>828</v>
+        <v>834</v>
       </c>
       <c r="B88" s="10" t="s">
         <v>371</v>
       </c>
       <c r="C88" s="10" t="s">
-        <v>829</v>
+        <v>835</v>
       </c>
       <c r="D88" s="10" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>830</v>
+        <v>836</v>
       </c>
       <c r="F88" s="10" t="s">
-        <v>831</v>
+        <v>837</v>
       </c>
       <c r="G88" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B88,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B88,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9566,22 +9688,22 @@
     </row>
     <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="9" t="s">
-        <v>832</v>
+        <v>838</v>
       </c>
       <c r="B89" s="10" t="s">
         <v>371</v>
       </c>
       <c r="C89" s="10" t="s">
-        <v>833</v>
+        <v>839</v>
       </c>
       <c r="D89" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>834</v>
+        <v>840</v>
       </c>
       <c r="F89" s="10" t="s">
-        <v>835</v>
+        <v>841</v>
       </c>
       <c r="G89" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B89,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B89,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9606,16 +9728,16 @@
         <v>376</v>
       </c>
       <c r="C90" s="10" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
       <c r="D90" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E90" s="10" t="s">
-        <v>837</v>
+        <v>843</v>
       </c>
       <c r="F90" s="10" t="s">
-        <v>838</v>
+        <v>844</v>
       </c>
       <c r="G90" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B90,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B90,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9634,22 +9756,22 @@
     </row>
     <row r="91" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="9" t="s">
-        <v>839</v>
+        <v>845</v>
       </c>
       <c r="B91" s="10" t="s">
         <v>382</v>
       </c>
       <c r="C91" s="10" t="s">
-        <v>840</v>
+        <v>846</v>
       </c>
       <c r="D91" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>841</v>
+        <v>847</v>
       </c>
       <c r="F91" s="10" t="s">
-        <v>842</v>
+        <v>848</v>
       </c>
       <c r="G91" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B91,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B91,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9668,22 +9790,22 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="9" t="s">
-        <v>843</v>
+        <v>849</v>
       </c>
       <c r="B92" s="10" t="s">
         <v>382</v>
       </c>
       <c r="C92" s="10" t="s">
-        <v>844</v>
+        <v>850</v>
       </c>
       <c r="D92" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E92" s="10" t="s">
-        <v>845</v>
+        <v>851</v>
       </c>
       <c r="F92" s="10" t="s">
-        <v>846</v>
+        <v>852</v>
       </c>
       <c r="G92" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B92,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B92,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9702,22 +9824,22 @@
     </row>
     <row r="93" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="9" t="s">
-        <v>847</v>
+        <v>853</v>
       </c>
       <c r="B93" s="10" t="s">
         <v>388</v>
       </c>
       <c r="C93" s="10" t="s">
-        <v>848</v>
+        <v>854</v>
       </c>
       <c r="D93" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="F93" s="10" t="s">
-        <v>849</v>
+        <v>855</v>
       </c>
       <c r="G93" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B93,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B93,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9736,22 +9858,22 @@
     </row>
     <row r="94" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="9" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="B94" s="10" t="s">
         <v>388</v>
       </c>
       <c r="C94" s="10" t="s">
-        <v>851</v>
+        <v>857</v>
       </c>
       <c r="D94" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E94" s="10" t="s">
-        <v>852</v>
+        <v>858</v>
       </c>
       <c r="F94" s="10" t="s">
-        <v>853</v>
+        <v>859</v>
       </c>
       <c r="G94" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B94,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B94,'Decide &amp; Next'!$A:$A,0)),""))</f>
@@ -9768,34 +9890,34 @@
       <c r="L94" s="12"/>
       <c r="M94" s="11"/>
     </row>
-    <row r="95" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="9" t="s">
-        <v>854</v>
+        <v>860</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>432</v>
+        <v>395</v>
       </c>
       <c r="C95" s="10" t="s">
-        <v>855</v>
+        <v>861</v>
       </c>
       <c r="D95" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>856</v>
+        <v>862</v>
       </c>
       <c r="F95" s="10" t="s">
-        <v>857</v>
+        <v>863</v>
       </c>
       <c r="G95" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B95,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B95,'Decide &amp; Next'!$A:$A,0)),""))</f>
-        <v>Done</v>
+        <v>Fixed</v>
       </c>
       <c r="H95" s="10" t="s">
         <v>21</v>
       </c>
       <c r="I95" s="11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="J95" s="11"/>
       <c r="K95" s="11"/>
@@ -9804,75 +9926,245 @@
     </row>
     <row r="96" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="9" t="s">
-        <v>858</v>
+        <v>864</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>439</v>
+        <v>395</v>
       </c>
       <c r="C96" s="10" t="s">
-        <v>859</v>
+        <v>865</v>
       </c>
       <c r="D96" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E96" s="10" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="F96" s="10" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="G96" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B96,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B96,'Decide &amp; Next'!$A:$A,0)),""))</f>
-        <v>Done</v>
+        <v>Fixed</v>
       </c>
       <c r="H96" s="10" t="s">
         <v>21</v>
       </c>
       <c r="I96" s="11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="J96" s="11"/>
       <c r="K96" s="11"/>
       <c r="L96" s="12"/>
       <c r="M96" s="11"/>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="9" t="s">
-        <v>862</v>
+        <v>868</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>443</v>
+        <v>395</v>
       </c>
       <c r="C97" s="10" t="s">
-        <v>863</v>
+        <v>869</v>
       </c>
       <c r="D97" s="10" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>845</v>
+        <v>870</v>
       </c>
       <c r="F97" s="10" t="s">
-        <v>864</v>
+        <v>871</v>
       </c>
       <c r="G97" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B97,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B97,'Decide &amp; Next'!$A:$A,0)),""))</f>
-        <v>Done</v>
+        <v>Fixed</v>
       </c>
       <c r="H97" s="10" t="s">
         <v>21</v>
       </c>
       <c r="I97" s="11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="J97" s="11"/>
       <c r="K97" s="11"/>
       <c r="L97" s="12"/>
       <c r="M97" s="11"/>
     </row>
+    <row r="98" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="9" t="s">
+        <v>872</v>
+      </c>
+      <c r="B98" s="10" t="s">
+        <v>395</v>
+      </c>
+      <c r="C98" s="10" t="s">
+        <v>873</v>
+      </c>
+      <c r="D98" s="10" t="s">
+        <v>499</v>
+      </c>
+      <c r="E98" s="10" t="s">
+        <v>874</v>
+      </c>
+      <c r="F98" s="10" t="s">
+        <v>875</v>
+      </c>
+      <c r="G98" s="15" t="str">
+        <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B98,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B98,'Decide &amp; Next'!$A:$A,0)),""))</f>
+        <v>Fixed</v>
+      </c>
+      <c r="H98" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="I98" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="J98" s="11"/>
+      <c r="K98" s="11"/>
+      <c r="L98" s="12"/>
+      <c r="M98" s="11"/>
+    </row>
+    <row r="99" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="9" t="s">
+        <v>876</v>
+      </c>
+      <c r="B99" s="10" t="s">
+        <v>395</v>
+      </c>
+      <c r="C99" s="10" t="s">
+        <v>877</v>
+      </c>
+      <c r="D99" s="10" t="s">
+        <v>508</v>
+      </c>
+      <c r="E99" s="10" t="s">
+        <v>878</v>
+      </c>
+      <c r="F99" s="10" t="s">
+        <v>879</v>
+      </c>
+      <c r="G99" s="15" t="str">
+        <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B99,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B99,'Decide &amp; Next'!$A:$A,0)),""))</f>
+        <v>Fixed</v>
+      </c>
+      <c r="H99" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="I99" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="J99" s="11"/>
+      <c r="K99" s="11"/>
+      <c r="L99" s="12"/>
+      <c r="M99" s="11"/>
+    </row>
+    <row r="100" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="9" t="s">
+        <v>880</v>
+      </c>
+      <c r="B100" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="C100" s="10" t="s">
+        <v>881</v>
+      </c>
+      <c r="D100" s="10" t="s">
+        <v>499</v>
+      </c>
+      <c r="E100" s="10" t="s">
+        <v>882</v>
+      </c>
+      <c r="F100" s="10" t="s">
+        <v>883</v>
+      </c>
+      <c r="G100" s="15" t="str">
+        <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B100,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B100,'Decide &amp; Next'!$A:$A,0)),""))</f>
+        <v>Done</v>
+      </c>
+      <c r="H100" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="I100" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="J100" s="11"/>
+      <c r="K100" s="11"/>
+      <c r="L100" s="12"/>
+      <c r="M100" s="11"/>
+    </row>
+    <row r="101" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="9" t="s">
+        <v>884</v>
+      </c>
+      <c r="B101" s="10" t="s">
+        <v>445</v>
+      </c>
+      <c r="C101" s="10" t="s">
+        <v>885</v>
+      </c>
+      <c r="D101" s="10" t="s">
+        <v>499</v>
+      </c>
+      <c r="E101" s="10" t="s">
+        <v>886</v>
+      </c>
+      <c r="F101" s="10" t="s">
+        <v>887</v>
+      </c>
+      <c r="G101" s="15" t="str">
+        <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B101,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B101,'Decide &amp; Next'!$A:$A,0)),""))</f>
+        <v>Done</v>
+      </c>
+      <c r="H101" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="I101" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="J101" s="11"/>
+      <c r="K101" s="11"/>
+      <c r="L101" s="12"/>
+      <c r="M101" s="11"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="9" t="s">
+        <v>888</v>
+      </c>
+      <c r="B102" s="10" t="s">
+        <v>449</v>
+      </c>
+      <c r="C102" s="10" t="s">
+        <v>889</v>
+      </c>
+      <c r="D102" s="10" t="s">
+        <v>499</v>
+      </c>
+      <c r="E102" s="10" t="s">
+        <v>851</v>
+      </c>
+      <c r="F102" s="10" t="s">
+        <v>890</v>
+      </c>
+      <c r="G102" s="15" t="str">
+        <f aca="false">IFERROR(INDEX(Fixes!$J:$J,MATCH(B102,Fixes!$A:$A,0)),IFERROR(INDEX('Decide &amp; Next'!$G:$G,MATCH(B102,'Decide &amp; Next'!$A:$A,0)),""))</f>
+        <v>Done</v>
+      </c>
+      <c r="H102" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="I102" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="J102" s="11"/>
+      <c r="K102" s="11"/>
+      <c r="L102" s="12"/>
+      <c r="M102" s="11"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M97"/>
-  <conditionalFormatting sqref="I2:I297">
+  <autoFilter ref="A1:M102"/>
+  <conditionalFormatting sqref="I2:I302">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$I2="Pass"</formula>
     </cfRule>
@@ -9886,7 +10178,7 @@
       <formula>$I2="Not run"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H297">
+  <conditionalFormatting sqref="H2:H302">
     <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>$H2="Pass"</formula>
     </cfRule>
@@ -9900,7 +10192,7 @@
       <formula>$H2="Not automated"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G297">
+  <conditionalFormatting sqref="G2:G302">
     <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>$G2="Fixed"</formula>
     </cfRule>
@@ -9915,11 +10207,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I2:I297" type="list">
+    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I2:I302" type="list">
       <formula1>"Not run,Pass,Fail,Partial"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D2:D297" type="list">
+    <dataValidation allowBlank="true" error="Pick a value from the list." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D2:D302" type="list">
       <formula1>"ADV-1234,ADV-5678,ADV-9012"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>